<commit_message>
docs: sync 3-bus case solution with Hadi Saadat textbook benchmark
</commit_message>
<xml_diff>
--- a/backend_api/sample_cases/power_flow_result_user_case3.xlsx
+++ b/backend_api/sample_cases/power_flow_result_user_case3.xlsx
@@ -471,10 +471,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>227.0966</v>
+        <v>218.4228</v>
       </c>
       <c r="E2" t="n">
-        <v>438.7575</v>
+        <v>140.8515</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -493,10 +493,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9540999999999999</v>
+        <v>0.9717</v>
       </c>
       <c r="C3" t="n">
-        <v>-3.1472</v>
+        <v>-2.6965</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -524,13 +524,13 @@
         <v>1.04</v>
       </c>
       <c r="C4" t="n">
-        <v>1.9205</v>
+        <v>-0.4988</v>
       </c>
       <c r="D4" t="n">
         <v>200</v>
       </c>
       <c r="E4" t="n">
-        <v>-131.9108</v>
+        <v>146.1769</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -613,22 +613,22 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>212.2215</v>
+        <v>179.3618</v>
       </c>
       <c r="D2" t="n">
-        <v>149.4431</v>
+        <v>118.7339</v>
       </c>
       <c r="E2" t="n">
-        <v>-200</v>
+        <v>-170.9684</v>
       </c>
       <c r="F2" t="n">
-        <v>-125</v>
+        <v>-101.9472</v>
       </c>
       <c r="G2" t="n">
-        <v>12.2215</v>
+        <v>8.3934</v>
       </c>
       <c r="H2" t="n">
-        <v>24.4431</v>
+        <v>16.7867</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -641,91 +641,60 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>212.2215</v>
+        <v>39.061</v>
       </c>
       <c r="D3" t="n">
-        <v>149.4431</v>
+        <v>22.1176</v>
       </c>
       <c r="E3" t="n">
-        <v>-200</v>
+        <v>-38.8783</v>
       </c>
       <c r="F3" t="n">
-        <v>-125</v>
+        <v>-21.5693</v>
       </c>
       <c r="G3" t="n">
-        <v>12.2215</v>
+        <v>0.1828</v>
       </c>
       <c r="H3" t="n">
-        <v>24.4431</v>
+        <v>0.5483</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Line 1-2</t>
+          <t>Line 1-3</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>-98.6733</v>
+        <v>-229.0316</v>
       </c>
       <c r="D4" t="n">
-        <v>69.9357</v>
+        <v>-148.0528</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>238.8783</v>
       </c>
       <c r="F4" t="n">
-        <v>-65.9554</v>
+        <v>167.7462</v>
       </c>
       <c r="G4" t="n">
-        <v>1.3267</v>
+        <v>9.8467</v>
       </c>
       <c r="H4" t="n">
-        <v>3.9802</v>
+        <v>19.6934</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Line 1-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" t="n">
-        <v>-98.6733</v>
-      </c>
-      <c r="D5" t="n">
-        <v>69.9357</v>
-      </c>
-      <c r="E5" t="n">
-        <v>100</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-65.9554</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1.3267</v>
-      </c>
-      <c r="H5" t="n">
-        <v>3.9802</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Line 1-3</t>
+          <t>Line 2-3</t>
         </is>
       </c>
     </row>
@@ -767,7 +736,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>427.097</v>
+        <v>418.423</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -782,7 +751,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>306.847</v>
+        <v>287.028</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -827,7 +796,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27.097</v>
+        <v>18.423</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -842,7 +811,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>56.847</v>
+        <v>37.028</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -904,7 +873,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2e-08</v>
+        <v>0</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>

</xml_diff>